<commit_message>
resolvendo problemas instancia chromed
</commit_message>
<xml_diff>
--- a/EmissaoCND/src/Reports/EmissaoCND.xlsx
+++ b/EmissaoCND/src/Reports/EmissaoCND.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\thiag\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\thiag\source\repos\EmissaoCND\EmissaoCND\src\Reports\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{36729192-6770-48D3-9C91-9FC1B58DB1C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{677F47AE-5BEC-4A1F-BBD9-4B5503229C8E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{64079876-B1A4-43E1-878F-AE8926165DA3}"/>
   </bookViews>
@@ -39,19 +39,28 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2" uniqueCount="2">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
   <si>
     <t>CNPJ</t>
   </si>
   <si>
     <t>STATUS</t>
   </si>
+  <si>
+    <t>Nome Empresa</t>
+  </si>
+  <si>
+    <t>4US COMPANY LTDA</t>
+  </si>
+  <si>
+    <t>83.527.101/0001-42</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -74,7 +83,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -97,14 +106,29 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -439,146 +463,186 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{99775ABA-A5CF-4B4F-8C3D-17A9B448E09F}">
-  <dimension ref="A1:B32"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <dimension ref="A1:C32"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="52.875" customWidth="1"/>
-    <col min="2" max="2" width="80.75" customWidth="1"/>
+    <col min="1" max="1" width="59.28515625" customWidth="1"/>
+    <col min="2" max="2" width="52.85546875" customWidth="1"/>
+    <col min="3" max="3" width="80.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2">
-      <c r="A2" s="2"/>
-      <c r="B2" s="2"/>
-    </row>
-    <row r="3" spans="1:2">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C2" s="2"/>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="2"/>
-      <c r="B3" s="2"/>
-    </row>
-    <row r="4" spans="1:2">
+      <c r="B3" s="3"/>
+      <c r="C3" s="2"/>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="2"/>
-      <c r="B4" s="2"/>
-    </row>
-    <row r="5" spans="1:2">
+      <c r="B4" s="3"/>
+      <c r="C4" s="2"/>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="2"/>
-      <c r="B5" s="2"/>
-    </row>
-    <row r="6" spans="1:2">
+      <c r="B5" s="3"/>
+      <c r="C5" s="2"/>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="2"/>
-      <c r="B6" s="2"/>
-    </row>
-    <row r="7" spans="1:2">
+      <c r="B6" s="3"/>
+      <c r="C6" s="2"/>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="2"/>
-      <c r="B7" s="2"/>
-    </row>
-    <row r="8" spans="1:2">
+      <c r="B7" s="3"/>
+      <c r="C7" s="2"/>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="2"/>
-      <c r="B8" s="2"/>
-    </row>
-    <row r="9" spans="1:2">
+      <c r="B8" s="3"/>
+      <c r="C8" s="2"/>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="2"/>
-      <c r="B9" s="2"/>
-    </row>
-    <row r="10" spans="1:2">
+      <c r="B9" s="3"/>
+      <c r="C9" s="2"/>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" s="2"/>
-      <c r="B10" s="2"/>
-    </row>
-    <row r="11" spans="1:2">
+      <c r="B10" s="3"/>
+      <c r="C10" s="2"/>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" s="2"/>
-      <c r="B11" s="2"/>
-    </row>
-    <row r="12" spans="1:2">
+      <c r="B11" s="3"/>
+      <c r="C11" s="2"/>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" s="2"/>
-      <c r="B12" s="2"/>
-    </row>
-    <row r="13" spans="1:2">
+      <c r="B12" s="3"/>
+      <c r="C12" s="2"/>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" s="2"/>
-      <c r="B13" s="2"/>
-    </row>
-    <row r="14" spans="1:2">
+      <c r="B13" s="3"/>
+      <c r="C13" s="2"/>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" s="2"/>
-      <c r="B14" s="2"/>
-    </row>
-    <row r="15" spans="1:2">
+      <c r="B14" s="3"/>
+      <c r="C14" s="2"/>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" s="2"/>
-      <c r="B15" s="2"/>
-    </row>
-    <row r="16" spans="1:2">
+      <c r="B15" s="3"/>
+      <c r="C15" s="2"/>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" s="2"/>
-      <c r="B16" s="2"/>
-    </row>
-    <row r="17" spans="1:2">
+      <c r="B16" s="3"/>
+      <c r="C16" s="2"/>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" s="2"/>
-      <c r="B17" s="2"/>
-    </row>
-    <row r="18" spans="1:2">
+      <c r="B17" s="3"/>
+      <c r="C17" s="2"/>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" s="2"/>
-      <c r="B18" s="2"/>
-    </row>
-    <row r="19" spans="1:2">
+      <c r="B18" s="3"/>
+      <c r="C18" s="2"/>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" s="2"/>
-      <c r="B19" s="2"/>
-    </row>
-    <row r="20" spans="1:2">
+      <c r="B19" s="3"/>
+      <c r="C19" s="2"/>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" s="2"/>
-      <c r="B20" s="2"/>
-    </row>
-    <row r="21" spans="1:2">
+      <c r="B20" s="3"/>
+      <c r="C20" s="2"/>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" s="2"/>
-      <c r="B21" s="2"/>
-    </row>
-    <row r="22" spans="1:2">
+      <c r="B21" s="3"/>
+      <c r="C21" s="2"/>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" s="2"/>
-      <c r="B22" s="2"/>
-    </row>
-    <row r="23" spans="1:2">
+      <c r="B22" s="3"/>
+      <c r="C22" s="2"/>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" s="2"/>
-      <c r="B23" s="2"/>
-    </row>
-    <row r="24" spans="1:2">
+      <c r="B23" s="3"/>
+      <c r="C23" s="2"/>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" s="2"/>
-      <c r="B24" s="2"/>
-    </row>
-    <row r="25" spans="1:2">
+      <c r="B24" s="3"/>
+      <c r="C24" s="2"/>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" s="2"/>
-      <c r="B25" s="2"/>
-    </row>
-    <row r="26" spans="1:2">
+      <c r="B25" s="3"/>
+      <c r="C25" s="2"/>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" s="2"/>
-      <c r="B26" s="2"/>
-    </row>
-    <row r="27" spans="1:2">
+      <c r="B26" s="3"/>
+      <c r="C26" s="2"/>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" s="2"/>
-      <c r="B27" s="2"/>
-    </row>
-    <row r="28" spans="1:2">
+      <c r="B27" s="3"/>
+      <c r="C27" s="2"/>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" s="2"/>
-      <c r="B28" s="2"/>
-    </row>
-    <row r="29" spans="1:2">
+      <c r="B28" s="3"/>
+      <c r="C28" s="2"/>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" s="2"/>
-      <c r="B29" s="2"/>
-    </row>
-    <row r="30" spans="1:2">
+      <c r="B29" s="3"/>
+      <c r="C29" s="2"/>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A30" s="2"/>
-      <c r="B30" s="2"/>
-    </row>
-    <row r="31" spans="1:2">
+      <c r="B30" s="3"/>
+      <c r="C30" s="2"/>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A31" s="2"/>
-      <c r="B31" s="2"/>
-    </row>
-    <row r="32" spans="1:2">
+      <c r="B31" s="3"/>
+      <c r="C31" s="2"/>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A32" s="2"/>
-      <c r="B32" s="2"/>
+      <c r="B32" s="3"/>
+      <c r="C32" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>